<commit_message>
Update MultiMap-Views.xlsx with new data and enhancements.
</commit_message>
<xml_diff>
--- a/printing/examples/MultiMap-Views.xlsx
+++ b/printing/examples/MultiMap-Views.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brent\Desktop\GIT\kirra-docs\printing\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{22BA9D15-B321-4CB7-9867-CC0FBD2F6F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D80BF08-1D20-403E-AFC9-C66F90D4C06B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-5600" windowWidth="38620" windowHeight="21100" xr2:uid="{B1B0B4BA-4EF6-4B6F-AE5E-EFA35A97AB33}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{B1B0B4BA-4EF6-4B6F-AE5E-EFA35A97AB33}"/>
   </bookViews>
   <sheets>
     <sheet name="Multi-Map-View" sheetId="1" r:id="rId1"/>
@@ -78,16 +78,16 @@
     <t>fx:mapView(v,8,rel,hid)</t>
   </si>
   <si>
-    <t>fx:mapView(v,15,slp)</t>
-  </si>
-  <si>
     <t>fx:legend(slp, v)</t>
   </si>
   <si>
-    <t>fx:mapView(v,15,rel)</t>
-  </si>
-  <si>
     <t>fx:legend(rel, v)</t>
+  </si>
+  <si>
+    <t>fx:mapView(r,150,rel)</t>
+  </si>
+  <si>
+    <t>fx:mapView(r,150,slp)</t>
   </si>
 </sst>
 </file>
@@ -138,12 +138,12 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -495,57 +495,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="2.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" ht="229.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" spans="1:5" ht="229.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
+      <c r="A3" s="1"/>
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="1"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" ht="229.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2"/>
-      <c r="B4" s="3" t="s">
+      <c r="A4" s="1"/>
+      <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="1"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5" ht="2.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2"/>
+      <c r="A5" s="1"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
-      <c r="E5" s="1"/>
+      <c r="E5" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -576,52 +576,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="2.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:6" ht="409.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" ht="409.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="1"/>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" ht="409.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6" ht="2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
-      <c r="F4" s="1"/>
+      <c r="F4" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>